<commit_message>
et ouai la team le halstead est la
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_By_William.xlsx
+++ b/mesures/TP_mesures_By_William.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="LOC" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="CC" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="halstead" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="95">
   <si>
     <t xml:space="preserve">Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -186,18 +187,140 @@
   </si>
   <si>
     <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Métriques de Halstead - iqsort0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opérateurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opérandes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mesures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opérateur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Occurrences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opérande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nt (opérateurs distincts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">void</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iqsort0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nt (occurrences d'opérateurs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">( )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">swap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nd (opérandes distincts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nd (occurrences d'opérandes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longueur N = Nt + Nd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vocabulaire n = nt + nd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{ }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volume = N * log2(n)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difficulté = (nt/2) * (Nd/nd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effort = Difficulté * Volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">++</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ ]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,6 +370,32 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -296,7 +445,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -334,6 +483,34 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1079,4 +1256,395 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <f aca="false">COUNTA(A5:A21)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <f aca="false">SUM(B5:B21)</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <f aca="false">COUNTA(D5:D12)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <f aca="false">SUM(E5:E12)</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <f aca="false">H5+H7</f>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <f aca="false">H4+H6</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <f aca="false">H8*LOG(H9,2)</f>
+        <v>390.083919941077</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <f aca="false">(H4/2)*(H7/H6)</f>
+        <v>38.25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="1"/>
+      <c r="G12" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <f aca="false">H11*H10</f>
+        <v>14920.7099377462</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="1"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
OMG LA REPONSE 7 LETS GOOOOOOOOOOOOOOOOOOOOOO
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_By_William.xlsx
+++ b/mesures/TP_mesures_By_William.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="98">
   <si>
     <t xml:space="preserve">Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -307,6 +307,15 @@
   </si>
   <si>
     <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question 7 - Validité des mesures de Halstead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selon la théorie de la mesure, la validité d'une métrique repose sur sa capacité à évaluer avec exactitude l'attribut ciblé. Elle doit traduire fidèlement la réalité empirique, par exemple en attribuant une valeur supérieure à un code reconnu comme plus complexe. De plus, sa définition se doit d'être parfaitement claire pour garantir la reproductibilité des résultats d'un évaluateur à l'autre. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutefois, les mesures de Halstead présentent des compteurs de base ambigus. Étant donné que deux personnes analysant exactement le même code peuvent aboutir à des résultats divergents, il est impossible de certifier que ces métriques quantifient correctement ce qu'elles sont censées représenter.</t>
   </si>
 </sst>
 </file>
@@ -320,7 +329,7 @@
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,6 +385,29 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <b val="true"/>
@@ -385,16 +417,10 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -445,7 +471,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -502,16 +528,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1263,7 +1297,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1328,17 +1362,17 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="13" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="1"/>
@@ -1351,17 +1385,17 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="13" t="n">
         <v>8</v>
       </c>
       <c r="C6" s="1"/>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="13" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="1"/>
@@ -1374,17 +1408,17 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="13" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="1"/>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="13" t="n">
         <v>7</v>
       </c>
       <c r="F7" s="1"/>
@@ -1397,17 +1431,17 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1"/>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="13" t="n">
         <v>4</v>
       </c>
       <c r="F8" s="1"/>
@@ -1420,17 +1454,17 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="13" t="n">
         <v>9</v>
       </c>
       <c r="C9" s="1"/>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="13" t="n">
         <v>6</v>
       </c>
       <c r="F9" s="1"/>
@@ -1443,79 +1477,79 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="1"/>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="13" t="n">
         <v>7</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="15" t="n">
+      <c r="H10" s="14" t="n">
         <f aca="false">H8*LOG(H9,2)</f>
         <v>390.083919941077</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="13" t="n">
         <v>8</v>
       </c>
       <c r="C11" s="1"/>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="13" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="H11" s="15" t="n">
+      <c r="H11" s="14" t="n">
         <f aca="false">(H4/2)*(H7/H6)</f>
         <v>38.25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B12" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1"/>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="13" t="n">
         <v>4</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="H12" s="16" t="n">
+      <c r="H12" s="15" t="n">
         <f aca="false">H11*H10</f>
         <v>14920.7099377462</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="1"/>
@@ -1526,10 +1560,10 @@
       <c r="H13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="1"/>
@@ -1540,10 +1574,10 @@
       <c r="H14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="1"/>
@@ -1554,10 +1588,10 @@
       <c r="H15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="1"/>
@@ -1568,10 +1602,10 @@
       <c r="H16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="1"/>
@@ -1582,10 +1616,10 @@
       <c r="H17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B18" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1"/>
@@ -1596,10 +1630,10 @@
       <c r="H18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B19" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C19" s="1"/>
@@ -1610,10 +1644,10 @@
       <c r="H19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="14" t="n">
+      <c r="B20" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C20" s="1"/>
@@ -1624,10 +1658,10 @@
       <c r="H20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="14" t="n">
+      <c r="B21" s="13" t="n">
         <v>2</v>
       </c>
       <c r="C21" s="1"/>
@@ -1637,8 +1671,59 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
     </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I22" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I24" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="18"/>
+      <c r="M24" s="18"/>
+      <c r="N24" s="18"/>
+      <c r="O24" s="18"/>
+      <c r="P24" s="18"/>
+    </row>
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I25" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="18"/>
+      <c r="P25" s="18"/>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="I22:P22"/>
+    <mergeCell ref="I23:P23"/>
+    <mergeCell ref="I24:P24"/>
+    <mergeCell ref="I25:P25"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
on continue sur la lancer l'équipe
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_By_William.xlsx
+++ b/mesures/TP_mesures_By_William.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LOC" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="CC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="halstead" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="albrecht" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="114">
   <si>
     <t xml:space="preserve">Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -316,6 +317,56 @@
   </si>
   <si>
     <t xml:space="preserve">Toutefois, les mesures de Halstead présentent des compteurs de base ambigus. Étant donné que deux personnes analysant exactement le même code peuvent aboutir à des résultats divergents, il est impossible de certifier que ces métriques quantifient correctement ce qu'elles sont censées représenter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score UFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catégorie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sous-total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrées externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3×4 + 4×3 + 6×1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorties externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4×0 + 5×2 + 7×1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requêtes externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3×7 + 4×0 + 6×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers internes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7×3 + 10×0 + 15×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5×0 + 7×5 + 10×2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
+Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
+Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
   </si>
 </sst>
 </file>
@@ -329,7 +380,7 @@
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -408,6 +459,27 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
     <font>
       <b val="true"/>
@@ -417,13 +489,13 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -434,6 +506,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2A6099"/>
+        <bgColor rgb="FF666699"/>
       </patternFill>
     </fill>
   </fills>
@@ -471,7 +549,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -536,15 +614,47 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -581,7 +691,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF2A6099"/>
       <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1732,4 +1842,124 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="24" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+    </row>
+    <row r="11" customFormat="false" ht="191.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:F11"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
et voila c jamais fini
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_By_William.xlsx
+++ b/mesures/TP_mesures_By_William.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="128">
   <si>
     <t xml:space="preserve">Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -367,6 +367,49 @@
     <t xml:space="preserve">Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
 Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
 Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poids (simple / moyen / difficile)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scores (simple / moyen / difficile)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 / 2 / 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 / 1 / 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1×1 + 2×1 + 4×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 / 3 / 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 / 1 / 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2×0 + 3×1 + 5×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 / 0 / 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1×0 + 2×0 + 4×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 / 5 / 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3×0 + 5×0 + 0×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+3 / 5 / 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3×0 + 5×0 + 8×0</t>
   </si>
 </sst>
 </file>
@@ -380,7 +423,7 @@
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -469,33 +512,14 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -512,6 +536,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF2A6099"/>
         <bgColor rgb="FF666699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -549,7 +579,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -626,36 +656,52 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1849,106 +1895,239 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="20" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="22" t="n">
+      <c r="C4" s="21" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="21" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="21" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="21" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="21" t="n">
         <v>55</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="24" t="n">
+      <c r="B9" s="21"/>
+      <c r="C9" s="22" t="n">
         <v>144</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="191.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+    </row>
+    <row r="16" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="26"/>
+      <c r="E16" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="E18" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="E19" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="29"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="30"/>
+      <c r="E22" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="F22" s="28"/>
+      <c r="G22" s="30" t="n">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
bababa le calcul MI
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_By_William.xlsx
+++ b/mesures/TP_mesures_By_William.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="LOC" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="CC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="halstead" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="albrecht" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="MI" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="135">
   <si>
     <t xml:space="preserve">Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -410,6 +411,27 @@
   </si>
   <si>
     <t xml:space="preserve">3×0 + 5×0 + 8×0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Index of maintenability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">171 - 5,2ln(HV) - 0,23CC - 16,2ln(LOC) + 50sin * sqrt(2,46COM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volume d’Halstead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complexité cyclomatique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre de lignes de code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pourcentage de lignes de code qui sont des commentaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">171 - 5,2 * ln(390,08) - 0,23 * 4 - 16,2 * ln(12) + 0 = 171 − 31,03 − 0,92 − 40,26 ≈ 98,80</t>
   </si>
 </sst>
 </file>
@@ -519,7 +541,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,13 +557,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2A6099"/>
-        <bgColor rgb="FF666699"/>
+        <bgColor rgb="FF3366FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5983B0"/>
+        <bgColor rgb="FF808080"/>
       </patternFill>
     </fill>
   </fills>
@@ -680,28 +708,28 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -761,7 +789,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -1996,6 +2024,10 @@
       <c r="E11" s="24"/>
       <c r="F11" s="24"/>
     </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
         <v>99</v>
@@ -2007,125 +2039,125 @@
         <v>115</v>
       </c>
       <c r="D16" s="26"/>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="20" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="G17" s="28" t="n">
+      <c r="G17" s="21" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="G18" s="28" t="n">
+      <c r="G18" s="21" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E19" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="28" t="n">
+      <c r="G19" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E20" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="F20" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="G20" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F21" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="G21" s="28" t="n">
+      <c r="G21" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="30"/>
-      <c r="E22" s="29" t="s">
+      <c r="A22" s="13"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="22"/>
+      <c r="E22" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="F22" s="28"/>
-      <c r="G22" s="30" t="n">
+      <c r="F22" s="21"/>
+      <c r="G22" s="22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2141,4 +2173,98 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="F9" s="30" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F10" s="30" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F11" s="30" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F12" s="30" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A16:F16"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
pwoooooooooooooooooooooooooooo l'ajout de COM et le calcul il est tous neuf c un folie
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_By_William.xlsx
+++ b/mesures/TP_mesures_By_William.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="140">
   <si>
     <t xml:space="preserve">Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -419,19 +419,58 @@
     <t xml:space="preserve">171 - 5,2ln(HV) - 0,23CC - 16,2ln(LOC) + 50sin * sqrt(2,46COM)</t>
   </si>
   <si>
-    <t xml:space="preserve">Volume d’Halstead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complexité cyclomatique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nombre de lignes de code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pourcentage de lignes de code qui sont des commentaires</t>
+    <t xml:space="preserve">Volume d’Halstead (HV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complexité cyclomatique (CC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre de lignes de code (LOC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pourcentage de lignes de code qui sont des commentaires (COM)</t>
   </si>
   <si>
     <t xml:space="preserve">171 - 5,2 * ln(390,08) - 0,23 * 4 - 16,2 * ln(12) + 0 = 171 − 31,03 − 0,92 − 40,26 ≈ 98,80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcul avec COM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,52 ( 13 /24 )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">171 - 5,2 * ln(390,08) - 0,23 * 4 - 16,2 * ln(12) + 50 * sin * sqrt(2,46 * 0,52 ) = 171 − 31,03 − 0,92 − 40,26 + 45,24  ≈ 144,04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On voit que le score est plus elevé avec les commentaires vraiment c une singerie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/*
+ * Auteur      : Prénom NOM
+ * Date        : 08/10/2026
+ * Description : QuickSort simplifié (Bentley et McIlroy, 1993).
+ *               Trie en place les n premiers éléments du tableau a,
+ *               par ordre croissant.
+ */
+void iqsort0 ( int *a , int n )
+{
+    int i , j ;
+    // Cas de base : un tableau de 0 ou 1 élément est déjà trié
+    if ( n &lt;=1)
+        return ;
+    // Partitionnement autour du pivot a[0] : j = indice du dernier élément &lt; pivot
+    for ( i = 1 , j = 0; i &lt; n ; i ++)
+    // Si a[i] est plus petit que le pivot, on l'ajoute à la zone de gauche
+        if ( a [ i ] &lt; a [0])
+            swap (++ j , i , a );
+    // Place le pivot à sa position définitive j
+    swap (0 , j , a );
+    // Tri récursif de la partie gauche (éléments &lt; pivot)
+    iqsort0 (a , j );
+    // Tri récursif de la partie droite (éléments &gt;= pivot)
+    iqsort0 ( a + j +1 , n -j -1);
+}</t>
   </si>
 </sst>
 </file>
@@ -607,7 +646,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -716,7 +755,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -725,11 +776,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2180,7 +2227,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2221,20 +2268,38 @@
       <c r="F9" s="30" t="s">
         <v>130</v>
       </c>
+      <c r="J9" s="30" t="n">
+        <v>390.08</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+      <c r="O9" s="29"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F10" s="30" t="s">
         <v>131</v>
       </c>
+      <c r="J10" s="30" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F11" s="30" t="s">
         <v>132</v>
       </c>
+      <c r="J11" s="30" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F12" s="30" t="s">
         <v>133</v>
+      </c>
+      <c r="J12" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2249,15 +2314,111 @@
       <c r="D16" s="29"/>
       <c r="E16" s="29"/>
       <c r="F16" s="29"/>
+      <c r="L16" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="M16" s="29"/>
+      <c r="N16" s="29"/>
+      <c r="O16" s="29"/>
+      <c r="P16" s="29"/>
+      <c r="Q16" s="29"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="F23" s="30" t="s">
+        <v>130</v>
+      </c>
+      <c r="J23" s="30" t="n">
+        <v>390.08</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F24" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="J24" s="30" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F25" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="J25" s="30" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F26" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="J26" s="30" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="10">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="L9:O9"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="L16:Q16"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A33:E33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>